<commit_message>
add kept and removed cells to xlsx
</commit_message>
<xml_diff>
--- a/Docs/Database.xlsx
+++ b/Docs/Database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RIC394\repos\APSIM.RegistrationSystem\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\APSIM.RegistrationSystem\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56518821-06FB-4480-BB50-0A3D80FB3E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E18CF9F6-B3A3-42E7-A7E2-DC9E13552492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{607743A3-7AB8-49E4-9650-AA4EF4C869F5}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{607743A3-7AB8-49E4-9650-AA4EF4C869F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="35">
   <si>
     <t>Users</t>
   </si>
@@ -138,6 +138,12 @@
   </si>
   <si>
     <t>AboveFortyMillion</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>n</t>
   </si>
 </sst>
 </file>
@@ -561,25 +567,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12DB3059-4014-4444-9DF4-89D9C302957D}">
   <dimension ref="A2:Q12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="26.26953125" customWidth="1"/>
-    <col min="15" max="15" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.21875" customWidth="1"/>
+    <col min="15" max="15" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
-    <col min="17" max="17" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -587,7 +593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
         <v>2</v>
@@ -635,7 +641,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="G4" t="s">
         <v>16</v>
       </c>
@@ -670,7 +676,42 @@
         <v>46506</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O5" t="s">
+        <v>34</v>
+      </c>
+      <c r="P5" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -684,7 +725,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -698,7 +739,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -712,7 +753,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -726,7 +767,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>31</v>
       </c>

</xml_diff>